<commit_message>
41 Elizabeth Ct package: light RE/MAX layout, subject facts, comp notes, pricing read, before-we-list; calculator light theme
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/p/41-elizabeth-ct-4b5cd4/41-elizabeth-ct-seller-net-proceeds.xlsx
+++ b/p/41-elizabeth-ct-4b5cd4/41-elizabeth-ct-seller-net-proceeds.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Net Proceeds" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">'Net Proceeds'!$A$1:$D$20</definedName>
+    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">'Net Proceeds'!$A$1:$D$21</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -23,12 +23,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="19">
   <si>
     <t xml:space="preserve">Seller Net Proceeds</t>
   </si>
   <si>
-    <t xml:space="preserve">41 Elizabeth Ct, Secaucus, NJ</t>
+    <t xml:space="preserve">41 Elizabeth Ct, Secaucus, NJ 07094</t>
   </si>
   <si>
     <t xml:space="preserve">Michael Gonnelli | The Gonnelli Group | RE/MAX Select | 201-240-8422</t>
@@ -37,10 +37,10 @@
     <t xml:space="preserve">Compensation rate</t>
   </si>
   <si>
-    <t xml:space="preserve">Partial RTF status</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Not confirmed; standard schedule shown</t>
+    <t xml:space="preserve">Reduced RTF eligibility confirmed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NO</t>
   </si>
   <si>
     <t xml:space="preserve">Sale Price</t>
@@ -58,10 +58,10 @@
     <t xml:space="preserve">Attorney Fee</t>
   </si>
   <si>
-    <t xml:space="preserve">Smoke Certificate</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Miscellaneous</t>
+    <t xml:space="preserve">Smoke and CO certificate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Other costs</t>
   </si>
   <si>
     <t xml:space="preserve">Total after costs</t>
@@ -73,10 +73,13 @@
     <t xml:space="preserve">Not provided</t>
   </si>
   <si>
-    <t xml:space="preserve">Proceeds Before Mortgage Payoff</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Transfer fee brackets: NJ Division of Taxation RTF schedule (over/under $350k), senior partial schedule, Graduated Percent Fee tiers from 7/10/2025. Estimates only.</t>
+    <t xml:space="preserve">Estimated Proceeds (Payoff Status Below)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Payoff status</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Blue cells are editable. Leave mortgage payoff as Not provided until known; enter 0 only if confirmed. Other liens, prorations and unlisted costs are excluded unless entered in Other costs. Reduced RTF requires confirmed eligibility with your attorney. Estimates only, not a closing statement. NJ RTF and July 2025 Graduated Percent Fee schedules apply.</t>
   </si>
 </sst>
 </file>
@@ -85,8 +88,8 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="General"/>
-    <numFmt numFmtId="165" formatCode="0.0%"/>
-    <numFmt numFmtId="166" formatCode="\$#,##0.00"/>
+    <numFmt numFmtId="165" formatCode="0.00##%"/>
+    <numFmt numFmtId="166" formatCode="\$#,##0.00;[RED]&quot;($&quot;#,##0.00\)"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -126,12 +129,18 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEAF1FA"/>
+        <bgColor rgb="FFCCFFFF"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -168,7 +177,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="10">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -177,7 +186,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -187,6 +204,14 @@
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -202,7 +227,110 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="FF000000"/>
+      <rgbColor rgb="FFEAF1FA"/>
+      <rgbColor rgb="FFFF0000"/>
+      <rgbColor rgb="FF00FF00"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF008000"/>
+      <rgbColor rgb="FF000080"/>
+      <rgbColor rgb="FF808000"/>
+      <rgbColor rgb="FF800080"/>
+      <rgbColor rgb="FF008080"/>
+      <rgbColor rgb="FFC0C0C0"/>
+      <rgbColor rgb="FF808080"/>
+      <rgbColor rgb="FF9999FF"/>
+      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FFFFFFCC"/>
+      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FF660066"/>
+      <rgbColor rgb="FFFF8080"/>
+      <rgbColor rgb="FF0066CC"/>
+      <rgbColor rgb="FFCCCCFF"/>
+      <rgbColor rgb="FF000080"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF800080"/>
+      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF008080"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FF00CCFF"/>
+      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FFCCFFCC"/>
+      <rgbColor rgb="FFFFFF99"/>
+      <rgbColor rgb="FF99CCFF"/>
+      <rgbColor rgb="FFFF99CC"/>
+      <rgbColor rgb="FFCC99FF"/>
+      <rgbColor rgb="FFFFCC99"/>
+      <rgbColor rgb="FF3366FF"/>
+      <rgbColor rgb="FF33CCCC"/>
+      <rgbColor rgb="FF99CC00"/>
+      <rgbColor rgb="FFFFCC00"/>
+      <rgbColor rgb="FFFF9900"/>
+      <rgbColor rgb="FFFF6600"/>
+      <rgbColor rgb="FF666699"/>
+      <rgbColor rgb="FF969696"/>
+      <rgbColor rgb="FF003366"/>
+      <rgbColor rgb="FF339966"/>
+      <rgbColor rgb="FF003300"/>
+      <rgbColor rgb="FF333300"/>
+      <rgbColor rgb="FF993300"/>
+      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FF333399"/>
+      <rgbColor rgb="FF333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>1504440</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>27000</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1" name="Image 1" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4581360" y="0"/>
+          <a:ext cx="1504440" cy="628200"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -385,11 +513,11 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="0" width="22"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -419,7 +547,7 @@
       <c r="A6" s="0" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="3" t="s">
         <v>5</v>
       </c>
     </row>
@@ -427,13 +555,13 @@
       <c r="A8" s="0" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="3" t="n">
+      <c r="B8" s="4" t="n">
         <v>750000</v>
       </c>
-      <c r="C8" s="3" t="n">
+      <c r="C8" s="4" t="n">
         <v>775000</v>
       </c>
-      <c r="D8" s="3" t="n">
+      <c r="D8" s="4" t="n">
         <v>800000</v>
       </c>
     </row>
@@ -441,16 +569,16 @@
       <c r="A9" s="0" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="3" t="n">
-        <f aca="false">IF(OR(NOT(ISNUMBER(B8)),B8&lt;0),NA(),ROUND(IF(B8&lt;=350000,ROUNDUP(MAX(0,MIN(B8,150000)-0)/500,0)*2+ROUNDUP(MAX(0,MIN(B8,200000)-150000)/500,0)*3.35+ROUNDUP(MAX(0,MIN(B8,350000)-200000)/500,0)*3.9,ROUNDUP(MAX(0,MIN(B8,150000)-0)/500,0)*2.9+ROUNDUP(MAX(0,MIN(B8,200000)-150000)/500,0)*4.25+ROUNDUP(MAX(0,MIN(B8,550000)-200000)/500,0)*4.8+ROUNDUP(MAX(0,MIN(B8,850000)-550000)/500,0)*5.3+ROUNDUP(MAX(0,MIN(B8,1000000)-850000)/500,0)*5.8+ROUNDUP(MAX(0,B8-1000000)/500,0)*6.05),2))</f>
+      <c r="B9" s="5" t="n">
+        <f aca="false">ROUND(IF(ROUND(B8,2)&lt;=350000,IF($B$6="YES",ROUNDUP(MAX(0,MIN(ROUND(B8,2),150000)-0)/500,0)*0.5+ROUNDUP(MAX(0,MIN(ROUND(B8,2),350000)-150000)/500,0)*1.25,ROUNDUP(MAX(0,MIN(ROUND(B8,2),150000)-0)/500,0)*2+ROUNDUP(MAX(0,MIN(ROUND(B8,2),200000)-150000)/500,0)*3.35+ROUNDUP(MAX(0,MIN(ROUND(B8,2),350000)-200000)/500,0)*3.9),IF($B$6="YES",ROUNDUP(MAX(0,MIN(ROUND(B8,2),150000)-0)/500,0)*1.4+ROUNDUP(MAX(0,MIN(ROUND(B8,2),550000)-150000)/500,0)*2.15+ROUNDUP(MAX(0,MIN(ROUND(B8,2),850000)-550000)/500,0)*2.65+ROUNDUP(MAX(0,MIN(ROUND(B8,2),1000000)-850000)/500,0)*3.15+ROUNDUP(MAX(0,ROUND(B8,2)-1000000)/500,0)*3.4,ROUNDUP(MAX(0,MIN(ROUND(B8,2),150000)-0)/500,0)*2.9+ROUNDUP(MAX(0,MIN(ROUND(B8,2),200000)-150000)/500,0)*4.25+ROUNDUP(MAX(0,MIN(ROUND(B8,2),550000)-200000)/500,0)*4.8+ROUNDUP(MAX(0,MIN(ROUND(B8,2),850000)-550000)/500,0)*5.3+ROUNDUP(MAX(0,MIN(ROUND(B8,2),1000000)-850000)/500,0)*5.8+ROUNDUP(MAX(0,ROUND(B8,2)-1000000)/500,0)*6.05)),2)</f>
         <v>6775</v>
       </c>
-      <c r="C9" s="3" t="n">
-        <f aca="false">IF(OR(NOT(ISNUMBER(C8)),C8&lt;0),NA(),ROUND(IF(C8&lt;=350000,ROUNDUP(MAX(0,MIN(C8,150000)-0)/500,0)*2+ROUNDUP(MAX(0,MIN(C8,200000)-150000)/500,0)*3.35+ROUNDUP(MAX(0,MIN(C8,350000)-200000)/500,0)*3.9,ROUNDUP(MAX(0,MIN(C8,150000)-0)/500,0)*2.9+ROUNDUP(MAX(0,MIN(C8,200000)-150000)/500,0)*4.25+ROUNDUP(MAX(0,MIN(C8,550000)-200000)/500,0)*4.8+ROUNDUP(MAX(0,MIN(C8,850000)-550000)/500,0)*5.3+ROUNDUP(MAX(0,MIN(C8,1000000)-850000)/500,0)*5.8+ROUNDUP(MAX(0,C8-1000000)/500,0)*6.05),2))</f>
+      <c r="C9" s="5" t="n">
+        <f aca="false">ROUND(IF(ROUND(C8,2)&lt;=350000,IF($B$6="YES",ROUNDUP(MAX(0,MIN(ROUND(C8,2),150000)-0)/500,0)*0.5+ROUNDUP(MAX(0,MIN(ROUND(C8,2),350000)-150000)/500,0)*1.25,ROUNDUP(MAX(0,MIN(ROUND(C8,2),150000)-0)/500,0)*2+ROUNDUP(MAX(0,MIN(ROUND(C8,2),200000)-150000)/500,0)*3.35+ROUNDUP(MAX(0,MIN(ROUND(C8,2),350000)-200000)/500,0)*3.9),IF($B$6="YES",ROUNDUP(MAX(0,MIN(ROUND(C8,2),150000)-0)/500,0)*1.4+ROUNDUP(MAX(0,MIN(ROUND(C8,2),550000)-150000)/500,0)*2.15+ROUNDUP(MAX(0,MIN(ROUND(C8,2),850000)-550000)/500,0)*2.65+ROUNDUP(MAX(0,MIN(ROUND(C8,2),1000000)-850000)/500,0)*3.15+ROUNDUP(MAX(0,ROUND(C8,2)-1000000)/500,0)*3.4,ROUNDUP(MAX(0,MIN(ROUND(C8,2),150000)-0)/500,0)*2.9+ROUNDUP(MAX(0,MIN(ROUND(C8,2),200000)-150000)/500,0)*4.25+ROUNDUP(MAX(0,MIN(ROUND(C8,2),550000)-200000)/500,0)*4.8+ROUNDUP(MAX(0,MIN(ROUND(C8,2),850000)-550000)/500,0)*5.3+ROUNDUP(MAX(0,MIN(ROUND(C8,2),1000000)-850000)/500,0)*5.8+ROUNDUP(MAX(0,ROUND(C8,2)-1000000)/500,0)*6.05)),2)</f>
         <v>7040</v>
       </c>
-      <c r="D9" s="3" t="n">
-        <f aca="false">IF(OR(NOT(ISNUMBER(D8)),D8&lt;0),NA(),ROUND(IF(D8&lt;=350000,ROUNDUP(MAX(0,MIN(D8,150000)-0)/500,0)*2+ROUNDUP(MAX(0,MIN(D8,200000)-150000)/500,0)*3.35+ROUNDUP(MAX(0,MIN(D8,350000)-200000)/500,0)*3.9,ROUNDUP(MAX(0,MIN(D8,150000)-0)/500,0)*2.9+ROUNDUP(MAX(0,MIN(D8,200000)-150000)/500,0)*4.25+ROUNDUP(MAX(0,MIN(D8,550000)-200000)/500,0)*4.8+ROUNDUP(MAX(0,MIN(D8,850000)-550000)/500,0)*5.3+ROUNDUP(MAX(0,MIN(D8,1000000)-850000)/500,0)*5.8+ROUNDUP(MAX(0,D8-1000000)/500,0)*6.05),2))</f>
+      <c r="D9" s="5" t="n">
+        <f aca="false">ROUND(IF(ROUND(D8,2)&lt;=350000,IF($B$6="YES",ROUNDUP(MAX(0,MIN(ROUND(D8,2),150000)-0)/500,0)*0.5+ROUNDUP(MAX(0,MIN(ROUND(D8,2),350000)-150000)/500,0)*1.25,ROUNDUP(MAX(0,MIN(ROUND(D8,2),150000)-0)/500,0)*2+ROUNDUP(MAX(0,MIN(ROUND(D8,2),200000)-150000)/500,0)*3.35+ROUNDUP(MAX(0,MIN(ROUND(D8,2),350000)-200000)/500,0)*3.9),IF($B$6="YES",ROUNDUP(MAX(0,MIN(ROUND(D8,2),150000)-0)/500,0)*1.4+ROUNDUP(MAX(0,MIN(ROUND(D8,2),550000)-150000)/500,0)*2.15+ROUNDUP(MAX(0,MIN(ROUND(D8,2),850000)-550000)/500,0)*2.65+ROUNDUP(MAX(0,MIN(ROUND(D8,2),1000000)-850000)/500,0)*3.15+ROUNDUP(MAX(0,ROUND(D8,2)-1000000)/500,0)*3.4,ROUNDUP(MAX(0,MIN(ROUND(D8,2),150000)-0)/500,0)*2.9+ROUNDUP(MAX(0,MIN(ROUND(D8,2),200000)-150000)/500,0)*4.25+ROUNDUP(MAX(0,MIN(ROUND(D8,2),550000)-200000)/500,0)*4.8+ROUNDUP(MAX(0,MIN(ROUND(D8,2),850000)-550000)/500,0)*5.3+ROUNDUP(MAX(0,MIN(ROUND(D8,2),1000000)-850000)/500,0)*5.8+ROUNDUP(MAX(0,ROUND(D8,2)-1000000)/500,0)*6.05)),2)</f>
         <v>7305</v>
       </c>
     </row>
@@ -458,16 +586,16 @@
       <c r="A10" s="0" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="3" t="n">
-        <f aca="false">IF(OR(NOT(ISNUMBER(B8)),B8&lt;0),NA(),ROUND(IF(B8&lt;=1000000,B8*0,IF(B8&lt;=2000000,B8*0.01,IF(B8&lt;=2500000,B8*0.02,IF(B8&lt;=3000000,B8*0.025,IF(B8&lt;=3500000,B8*0.03,B8*0.035))))),2))</f>
+      <c r="B10" s="5" t="n">
+        <f aca="false">ROUND(ROUND(B8,2)*IF(ROUND(B8,2)&lt;=1000000,0,IF(ROUND(B8,2)&lt;=2000000,0.01,IF(ROUND(B8,2)&lt;=2500000,0.02,IF(ROUND(B8,2)&lt;=3000000,0.025,IF(ROUND(B8,2)&lt;=3500000,0.03,0.035))))),2)</f>
         <v>0</v>
       </c>
-      <c r="C10" s="3" t="n">
-        <f aca="false">IF(OR(NOT(ISNUMBER(C8)),C8&lt;0),NA(),ROUND(IF(C8&lt;=1000000,C8*0,IF(C8&lt;=2000000,C8*0.01,IF(C8&lt;=2500000,C8*0.02,IF(C8&lt;=3000000,C8*0.025,IF(C8&lt;=3500000,C8*0.03,C8*0.035))))),2))</f>
+      <c r="C10" s="5" t="n">
+        <f aca="false">ROUND(ROUND(C8,2)*IF(ROUND(C8,2)&lt;=1000000,0,IF(ROUND(C8,2)&lt;=2000000,0.01,IF(ROUND(C8,2)&lt;=2500000,0.02,IF(ROUND(C8,2)&lt;=3000000,0.025,IF(ROUND(C8,2)&lt;=3500000,0.03,0.035))))),2)</f>
         <v>0</v>
       </c>
-      <c r="D10" s="3" t="n">
-        <f aca="false">IF(OR(NOT(ISNUMBER(D8)),D8&lt;0),NA(),ROUND(IF(D8&lt;=1000000,D8*0,IF(D8&lt;=2000000,D8*0.01,IF(D8&lt;=2500000,D8*0.02,IF(D8&lt;=3000000,D8*0.025,IF(D8&lt;=3500000,D8*0.03,D8*0.035))))),2))</f>
+      <c r="D10" s="5" t="n">
+        <f aca="false">ROUND(ROUND(D8,2)*IF(ROUND(D8,2)&lt;=1000000,0,IF(ROUND(D8,2)&lt;=2000000,0.01,IF(ROUND(D8,2)&lt;=2500000,0.02,IF(ROUND(D8,2)&lt;=3000000,0.025,IF(ROUND(D8,2)&lt;=3500000,0.03,0.035))))),2)</f>
         <v>0</v>
       </c>
     </row>
@@ -475,16 +603,16 @@
       <c r="A11" s="0" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="3" t="n">
-        <f aca="false">IF(OR(NOT(ISNUMBER(B8)),B8&lt;0),NA(),ROUND($B$5*B8,2))</f>
+      <c r="B11" s="5" t="n">
+        <f aca="false">ROUND($B$5*ROUND(B8,2),2)</f>
         <v>30000</v>
       </c>
-      <c r="C11" s="3" t="n">
-        <f aca="false">IF(OR(NOT(ISNUMBER(C8)),C8&lt;0),NA(),ROUND($B$5*C8,2))</f>
+      <c r="C11" s="5" t="n">
+        <f aca="false">ROUND($B$5*ROUND(C8,2),2)</f>
         <v>31000</v>
       </c>
-      <c r="D11" s="3" t="n">
-        <f aca="false">IF(OR(NOT(ISNUMBER(D8)),D8&lt;0),NA(),ROUND($B$5*D8,2))</f>
+      <c r="D11" s="5" t="n">
+        <f aca="false">ROUND($B$5*ROUND(D8,2),2)</f>
         <v>32000</v>
       </c>
     </row>
@@ -492,13 +620,13 @@
       <c r="A12" s="0" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="3" t="n">
+      <c r="B12" s="4" t="n">
         <v>1500</v>
       </c>
-      <c r="C12" s="3" t="n">
+      <c r="C12" s="4" t="n">
         <v>1500</v>
       </c>
-      <c r="D12" s="3" t="n">
+      <c r="D12" s="4" t="n">
         <v>1500</v>
       </c>
     </row>
@@ -506,13 +634,13 @@
       <c r="A13" s="0" t="s">
         <v>11</v>
       </c>
-      <c r="B13" s="3" t="n">
+      <c r="B13" s="4" t="n">
         <v>200</v>
       </c>
-      <c r="C13" s="3" t="n">
+      <c r="C13" s="4" t="n">
         <v>200</v>
       </c>
-      <c r="D13" s="3" t="n">
+      <c r="D13" s="4" t="n">
         <v>200</v>
       </c>
     </row>
@@ -520,30 +648,30 @@
       <c r="A14" s="0" t="s">
         <v>12</v>
       </c>
-      <c r="B14" s="3" t="n">
+      <c r="B14" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="C14" s="3" t="n">
+      <c r="C14" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="D14" s="3" t="n">
+      <c r="D14" s="4" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="4" t="s">
+      <c r="A15" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B15" s="3" t="n">
-        <f aca="false">ROUND(B8-SUM(B9:B14),2)</f>
+      <c r="B15" s="5" t="n">
+        <f aca="false">ROUND(ROUND(B8,2)-SUM(B9:B11)-ROUND(B12,2)-ROUND(B13,2)-ROUND(B14,2),2)</f>
         <v>711525</v>
       </c>
-      <c r="C15" s="3" t="n">
-        <f aca="false">ROUND(C8-SUM(C9:C14),2)</f>
+      <c r="C15" s="5" t="n">
+        <f aca="false">ROUND(ROUND(C8,2)-SUM(C9:C11)-ROUND(C12,2)-ROUND(C13,2)-ROUND(C14,2),2)</f>
         <v>735260</v>
       </c>
-      <c r="D15" s="3" t="n">
-        <f aca="false">ROUND(D8-SUM(D9:D14),2)</f>
+      <c r="D15" s="5" t="n">
+        <f aca="false">ROUND(ROUND(D8,2)-SUM(D9:D11)-ROUND(D12,2)-ROUND(D13,2)-ROUND(D14,2),2)</f>
         <v>758995</v>
       </c>
     </row>
@@ -551,54 +679,109 @@
       <c r="A16" s="0" t="s">
         <v>14</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="B16" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="C16" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="D16" s="3" t="s">
+      <c r="D16" s="7" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="4" t="s">
+      <c r="A17" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="B17" s="3" t="n">
-        <f aca="false">B15</f>
+      <c r="B17" s="5" t="n">
+        <f aca="false">ROUND(B15-IF(ISNUMBER(B16),ROUND(B16,2),0),2)</f>
         <v>711525</v>
       </c>
-      <c r="C17" s="3" t="n">
-        <f aca="false">C15</f>
+      <c r="C17" s="5" t="n">
+        <f aca="false">ROUND(C15-IF(ISNUMBER(C16),ROUND(C16,2),0),2)</f>
         <v>735260</v>
       </c>
-      <c r="D17" s="3" t="n">
-        <f aca="false">D15</f>
+      <c r="D17" s="5" t="n">
+        <f aca="false">ROUND(D15-IF(ISNUMBER(D16),ROUND(D16,2),0),2)</f>
         <v>758995</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="5" t="s">
+    <row r="18" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="0" t="s">
         <v>17</v>
       </c>
-      <c r="B19" s="5"/>
-      <c r="C19" s="5"/>
-      <c r="D19" s="5"/>
+      <c r="B18" s="8" t="str">
+        <f aca="false">IF(ISNUMBER(B16),"After entered payoff","Before payoff (not provided)")</f>
+        <v>Before payoff (not provided)</v>
+      </c>
+      <c r="C18" s="8" t="str">
+        <f aca="false">IF(ISNUMBER(C16),"After entered payoff","Before payoff (not provided)")</f>
+        <v>Before payoff (not provided)</v>
+      </c>
+      <c r="D18" s="8" t="str">
+        <f aca="false">IF(ISNUMBER(D16),"After entered payoff","Before payoff (not provided)")</f>
+        <v>Before payoff (not provided)</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B19" s="9"/>
+      <c r="C19" s="9"/>
+      <c r="D19" s="9"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="5"/>
-      <c r="B20" s="5"/>
-      <c r="C20" s="5"/>
-      <c r="D20" s="5"/>
+      <c r="A20" s="9"/>
+      <c r="B20" s="9"/>
+      <c r="C20" s="9"/>
+      <c r="D20" s="9"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="9"/>
+      <c r="B21" s="9"/>
+      <c r="C21" s="9"/>
+      <c r="D21" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A19:D20"/>
+    <mergeCell ref="A19:D21"/>
   </mergeCells>
-  <dataValidations count="1">
-    <dataValidation allowBlank="false" error="Enter a non-negative sale price as a number." errorStyle="stop" errorTitle="Invalid sale price" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="B8:D8" type="custom">
-      <formula1>AND(ISNUMBER(B8),B8&gt;=0)</formula1>
+  <dataValidations count="9">
+    <dataValidation allowBlank="false" error="Enter a nonnegative amount." errorStyle="stop" operator="greaterThanOrEqual" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="B12:D14" type="decimal">
+      <formula1>0</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" error="Enter a sale price greater than zero." errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="B8" type="custom">
+      <formula1>AND(ISNUMBER(B8),ROUND(B8,2)&gt;0)</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" error="Enter a nonnegative payoff, or leave Not provided." errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="B16" type="custom">
+      <formula1>OR(B16="",B16="Not provided",AND(ISNUMBER(B16),B16&gt;=0))</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" error="Enter a sale price greater than zero." errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="C8" type="custom">
+      <formula1>AND(ISNUMBER(C8),ROUND(C8,2)&gt;0)</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" error="Enter a nonnegative payoff, or leave Not provided." errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="C16" type="custom">
+      <formula1>OR(C16="",C16="Not provided",AND(ISNUMBER(C16),C16&gt;=0))</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" error="Enter a sale price greater than zero." errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D8" type="custom">
+      <formula1>AND(ISNUMBER(D8),ROUND(D8,2)&gt;0)</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" error="Enter a nonnegative payoff, or leave Not provided." errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D16" type="custom">
+      <formula1>OR(D16="",D16="Not provided",AND(ISNUMBER(D16),D16&gt;=0))</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="B5" type="decimal">
+      <formula1>0</formula1>
+      <formula2>1</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="B6" type="list">
+      <formula1>"YES,NO"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -609,5 +792,6 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>